<commit_message>
Intermediate commit for reporting changes
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD20EB5B-36E2-4931-A02B-2BDAC4C4D805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD008B7-8B5C-4AAD-A923-959771D95CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1275" windowWidth="16575" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="1005" windowWidth="22125" windowHeight="13800" tabRatio="750" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7972" uniqueCount="1179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7862" uniqueCount="1163">
   <si>
     <t>;</t>
   </si>
@@ -3745,54 +3745,6 @@
   </si>
   <si>
     <t>09/15/25 - SAC - toggled off SysAvail for '22 VCHP Compliance Option system (gh dev #458)</t>
-  </si>
-  <si>
-    <t>NRMF 2025 ACM Table 47: HPWH System MMV (master mixing valve) Correction Factor</t>
-  </si>
-  <si>
-    <t>TABLE  T24MFDHW_CHPWH_MMVCorrectionFactor</t>
-  </si>
-  <si>
-    <t>SystemDescrip</t>
-  </si>
-  <si>
-    <t>OutletReturnDT</t>
-  </si>
-  <si>
-    <t>&lt;7</t>
-  </si>
-  <si>
-    <t>MPassInteg</t>
-  </si>
-  <si>
-    <t>Digital</t>
-  </si>
-  <si>
-    <t>MMVType</t>
-  </si>
-  <si>
-    <t>Mechanical</t>
-  </si>
-  <si>
-    <t>CorrectFactor</t>
-  </si>
-  <si>
-    <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>SPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>MPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>SPassPrim-SResist</t>
-  </si>
-  <si>
-    <t>SPassPrim-Parallel</t>
-  </si>
-  <si>
-    <t>08/01/26 - SAC - added T24MFDHW_CHPWH_MMVCorrectionFactor table (dev #942)</t>
   </si>
 </sst>
 </file>
@@ -4476,7 +4428,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4998,21 +4950,6 @@
     <xf numFmtId="0" fontId="11" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75191,14 +75128,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="20.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -75241,9 +75172,6 @@
       </c>
       <c r="B5" t="s">
         <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75514,602 +75442,6 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="145" t="s">
-        <v>1164</v>
-      </c>
-      <c r="C34" s="145"/>
-      <c r="D34" s="146"/>
-      <c r="E34" s="146"/>
-      <c r="F34" s="146"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D35" s="229" t="s">
-        <v>1165</v>
-      </c>
-      <c r="E35" s="147" t="s">
-        <v>1166</v>
-      </c>
-      <c r="F35" s="229" t="s">
-        <v>1170</v>
-      </c>
-      <c r="G35" s="148" t="s">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C36" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D36" s="230" t="s">
-        <v>1168</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F36" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G36" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D37" s="232" t="str">
-        <f>D36</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F37" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D38" s="232" t="str">
-        <f t="shared" ref="D38:D41" si="0">D37</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F38" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G38" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C39" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D39" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F39" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G39" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D40" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F40" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G40" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D41" s="233" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E41" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F41" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C42" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D42" s="230" t="s">
-        <v>1174</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F42" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G42" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C43" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D43" s="232" t="str">
-        <f>D42</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F43" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G43" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C44" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D44" s="232" t="str">
-        <f t="shared" ref="D44:D47" si="1">D43</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F44" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G44" s="1">
-        <v>1.1399999999999999</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C45" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D45" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F45" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C46" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D46" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F46" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G46" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C47" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D47" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E47" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F47" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.0900000000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C48" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D48" s="230" t="s">
-        <v>1175</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F48" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G48" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C49" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D49" s="232" t="str">
-        <f>D48</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F49" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G49" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C50" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D50" s="232" t="str">
-        <f t="shared" ref="D50:D53" si="2">D49</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F50" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G50" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C51" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D51" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F51" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G51" s="1">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C52" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D52" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F52" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G52" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C53" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D53" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E53" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F53" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C54" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D54" s="230" t="s">
-        <v>1176</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F54" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G54" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C55" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D55" s="232" t="str">
-        <f>D54</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F55" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G55" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D56" s="232" t="str">
-        <f t="shared" ref="D56:D59" si="3">D55</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F56" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G56" s="1">
-        <v>1.08</v>
-      </c>
-    </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D57" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F57" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G57" s="1">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F58" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G58" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E59" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F59" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C60" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D60" s="230" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F60" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G60" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C61" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D61" s="232" t="str">
-        <f>D60</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F61" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G61" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C62" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D62" s="232" t="str">
-        <f t="shared" ref="D62:D65" si="4">D61</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F62" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G62" s="1">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C63" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D63" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F63" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G63" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C64" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D64" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F64" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C65" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D65" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E65" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F65" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G65" s="22">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F66" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G66" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revised Altered Standard Design Constructions for E+A+A - Wd Wall 2x4 and 2x6 to mirror 160.1(c)3.
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD20EB5B-36E2-4931-A02B-2BDAC4C4D805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD008B7-8B5C-4AAD-A923-959771D95CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1275" windowWidth="16575" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="1005" windowWidth="22125" windowHeight="13800" tabRatio="750" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7972" uniqueCount="1179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7862" uniqueCount="1163">
   <si>
     <t>;</t>
   </si>
@@ -3745,54 +3745,6 @@
   </si>
   <si>
     <t>09/15/25 - SAC - toggled off SysAvail for '22 VCHP Compliance Option system (gh dev #458)</t>
-  </si>
-  <si>
-    <t>NRMF 2025 ACM Table 47: HPWH System MMV (master mixing valve) Correction Factor</t>
-  </si>
-  <si>
-    <t>TABLE  T24MFDHW_CHPWH_MMVCorrectionFactor</t>
-  </si>
-  <si>
-    <t>SystemDescrip</t>
-  </si>
-  <si>
-    <t>OutletReturnDT</t>
-  </si>
-  <si>
-    <t>&lt;7</t>
-  </si>
-  <si>
-    <t>MPassInteg</t>
-  </si>
-  <si>
-    <t>Digital</t>
-  </si>
-  <si>
-    <t>MMVType</t>
-  </si>
-  <si>
-    <t>Mechanical</t>
-  </si>
-  <si>
-    <t>CorrectFactor</t>
-  </si>
-  <si>
-    <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>SPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>MPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>SPassPrim-SResist</t>
-  </si>
-  <si>
-    <t>SPassPrim-Parallel</t>
-  </si>
-  <si>
-    <t>08/01/26 - SAC - added T24MFDHW_CHPWH_MMVCorrectionFactor table (dev #942)</t>
   </si>
 </sst>
 </file>
@@ -4476,7 +4428,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4998,21 +4950,6 @@
     <xf numFmtId="0" fontId="11" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75191,14 +75128,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="20.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -75241,9 +75172,6 @@
       </c>
       <c r="B5" t="s">
         <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75514,602 +75442,6 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="145" t="s">
-        <v>1164</v>
-      </c>
-      <c r="C34" s="145"/>
-      <c r="D34" s="146"/>
-      <c r="E34" s="146"/>
-      <c r="F34" s="146"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D35" s="229" t="s">
-        <v>1165</v>
-      </c>
-      <c r="E35" s="147" t="s">
-        <v>1166</v>
-      </c>
-      <c r="F35" s="229" t="s">
-        <v>1170</v>
-      </c>
-      <c r="G35" s="148" t="s">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C36" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D36" s="230" t="s">
-        <v>1168</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F36" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G36" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D37" s="232" t="str">
-        <f>D36</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F37" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D38" s="232" t="str">
-        <f t="shared" ref="D38:D41" si="0">D37</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F38" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G38" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C39" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D39" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F39" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G39" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D40" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F40" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G40" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D41" s="233" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E41" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F41" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C42" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D42" s="230" t="s">
-        <v>1174</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F42" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G42" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C43" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D43" s="232" t="str">
-        <f>D42</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F43" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G43" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C44" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D44" s="232" t="str">
-        <f t="shared" ref="D44:D47" si="1">D43</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F44" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G44" s="1">
-        <v>1.1399999999999999</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C45" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D45" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F45" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C46" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D46" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F46" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G46" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C47" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D47" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E47" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F47" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.0900000000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C48" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D48" s="230" t="s">
-        <v>1175</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F48" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G48" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C49" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D49" s="232" t="str">
-        <f>D48</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F49" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G49" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C50" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D50" s="232" t="str">
-        <f t="shared" ref="D50:D53" si="2">D49</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F50" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G50" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C51" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D51" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F51" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G51" s="1">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C52" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D52" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F52" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G52" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C53" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D53" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E53" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F53" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C54" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D54" s="230" t="s">
-        <v>1176</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F54" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G54" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C55" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D55" s="232" t="str">
-        <f>D54</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F55" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G55" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D56" s="232" t="str">
-        <f t="shared" ref="D56:D59" si="3">D55</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F56" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G56" s="1">
-        <v>1.08</v>
-      </c>
-    </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D57" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F57" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G57" s="1">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F58" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G58" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E59" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F59" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C60" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D60" s="230" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F60" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G60" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C61" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D61" s="232" t="str">
-        <f>D60</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F61" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G61" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C62" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D62" s="232" t="str">
-        <f t="shared" ref="D62:D65" si="4">D61</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F62" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G62" s="1">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C63" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D63" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F63" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G63" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C64" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D64" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F64" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C65" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D65" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E65" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F65" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G65" s="22">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F66" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G66" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add validation for “Exclude from Gross Floor Area” spaces set as Directly Conditioned Fixes #971 Add error check for "Exclude from Gross Floor Area" spaces marked as directly conditioned
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD20EB5B-36E2-4931-A02B-2BDAC4C4D805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD008B7-8B5C-4AAD-A923-959771D95CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1275" windowWidth="16575" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="1005" windowWidth="22125" windowHeight="13800" tabRatio="750" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7972" uniqueCount="1179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7862" uniqueCount="1163">
   <si>
     <t>;</t>
   </si>
@@ -3745,54 +3745,6 @@
   </si>
   <si>
     <t>09/15/25 - SAC - toggled off SysAvail for '22 VCHP Compliance Option system (gh dev #458)</t>
-  </si>
-  <si>
-    <t>NRMF 2025 ACM Table 47: HPWH System MMV (master mixing valve) Correction Factor</t>
-  </si>
-  <si>
-    <t>TABLE  T24MFDHW_CHPWH_MMVCorrectionFactor</t>
-  </si>
-  <si>
-    <t>SystemDescrip</t>
-  </si>
-  <si>
-    <t>OutletReturnDT</t>
-  </si>
-  <si>
-    <t>&lt;7</t>
-  </si>
-  <si>
-    <t>MPassInteg</t>
-  </si>
-  <si>
-    <t>Digital</t>
-  </si>
-  <si>
-    <t>MMVType</t>
-  </si>
-  <si>
-    <t>Mechanical</t>
-  </si>
-  <si>
-    <t>CorrectFactor</t>
-  </si>
-  <si>
-    <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>SPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>MPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>SPassPrim-SResist</t>
-  </si>
-  <si>
-    <t>SPassPrim-Parallel</t>
-  </si>
-  <si>
-    <t>08/01/26 - SAC - added T24MFDHW_CHPWH_MMVCorrectionFactor table (dev #942)</t>
   </si>
 </sst>
 </file>
@@ -4476,7 +4428,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4998,21 +4950,6 @@
     <xf numFmtId="0" fontId="11" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75191,14 +75128,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="20.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -75241,9 +75172,6 @@
       </c>
       <c r="B5" t="s">
         <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75514,602 +75442,6 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="145" t="s">
-        <v>1164</v>
-      </c>
-      <c r="C34" s="145"/>
-      <c r="D34" s="146"/>
-      <c r="E34" s="146"/>
-      <c r="F34" s="146"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D35" s="229" t="s">
-        <v>1165</v>
-      </c>
-      <c r="E35" s="147" t="s">
-        <v>1166</v>
-      </c>
-      <c r="F35" s="229" t="s">
-        <v>1170</v>
-      </c>
-      <c r="G35" s="148" t="s">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C36" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D36" s="230" t="s">
-        <v>1168</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F36" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G36" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D37" s="232" t="str">
-        <f>D36</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F37" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D38" s="232" t="str">
-        <f t="shared" ref="D38:D41" si="0">D37</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F38" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G38" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C39" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D39" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F39" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G39" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D40" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F40" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G40" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D41" s="233" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E41" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F41" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C42" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D42" s="230" t="s">
-        <v>1174</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F42" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G42" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C43" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D43" s="232" t="str">
-        <f>D42</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F43" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G43" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C44" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D44" s="232" t="str">
-        <f t="shared" ref="D44:D47" si="1">D43</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F44" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G44" s="1">
-        <v>1.1399999999999999</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C45" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D45" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F45" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C46" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D46" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F46" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G46" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C47" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D47" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E47" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F47" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.0900000000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C48" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D48" s="230" t="s">
-        <v>1175</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F48" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G48" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C49" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D49" s="232" t="str">
-        <f>D48</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F49" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G49" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C50" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D50" s="232" t="str">
-        <f t="shared" ref="D50:D53" si="2">D49</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F50" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G50" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C51" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D51" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F51" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G51" s="1">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C52" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D52" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F52" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G52" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C53" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D53" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E53" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F53" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C54" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D54" s="230" t="s">
-        <v>1176</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F54" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G54" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C55" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D55" s="232" t="str">
-        <f>D54</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F55" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G55" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D56" s="232" t="str">
-        <f t="shared" ref="D56:D59" si="3">D55</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F56" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G56" s="1">
-        <v>1.08</v>
-      </c>
-    </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D57" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F57" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G57" s="1">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F58" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G58" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E59" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F59" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C60" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D60" s="230" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F60" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G60" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C61" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D61" s="232" t="str">
-        <f>D60</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F61" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G61" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C62" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D62" s="232" t="str">
-        <f t="shared" ref="D62:D65" si="4">D61</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F62" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G62" s="1">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C63" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D63" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F63" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G63" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C64" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D64" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F64" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C65" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D65" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E65" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F65" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G65" s="22">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F66" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G66" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added wlFUA loss adjustment gate
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD20EB5B-36E2-4931-A02B-2BDAC4C4D805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD008B7-8B5C-4AAD-A923-959771D95CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1275" windowWidth="16575" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="1005" windowWidth="22125" windowHeight="13800" tabRatio="750" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7972" uniqueCount="1179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7862" uniqueCount="1163">
   <si>
     <t>;</t>
   </si>
@@ -3745,54 +3745,6 @@
   </si>
   <si>
     <t>09/15/25 - SAC - toggled off SysAvail for '22 VCHP Compliance Option system (gh dev #458)</t>
-  </si>
-  <si>
-    <t>NRMF 2025 ACM Table 47: HPWH System MMV (master mixing valve) Correction Factor</t>
-  </si>
-  <si>
-    <t>TABLE  T24MFDHW_CHPWH_MMVCorrectionFactor</t>
-  </si>
-  <si>
-    <t>SystemDescrip</t>
-  </si>
-  <si>
-    <t>OutletReturnDT</t>
-  </si>
-  <si>
-    <t>&lt;7</t>
-  </si>
-  <si>
-    <t>MPassInteg</t>
-  </si>
-  <si>
-    <t>Digital</t>
-  </si>
-  <si>
-    <t>MMVType</t>
-  </si>
-  <si>
-    <t>Mechanical</t>
-  </si>
-  <si>
-    <t>CorrectFactor</t>
-  </si>
-  <si>
-    <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>SPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>MPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>SPassPrim-SResist</t>
-  </si>
-  <si>
-    <t>SPassPrim-Parallel</t>
-  </si>
-  <si>
-    <t>08/01/26 - SAC - added T24MFDHW_CHPWH_MMVCorrectionFactor table (dev #942)</t>
   </si>
 </sst>
 </file>
@@ -4476,7 +4428,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4998,21 +4950,6 @@
     <xf numFmtId="0" fontId="11" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75191,14 +75128,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="20.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -75241,9 +75172,6 @@
       </c>
       <c r="B5" t="s">
         <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75514,602 +75442,6 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="145" t="s">
-        <v>1164</v>
-      </c>
-      <c r="C34" s="145"/>
-      <c r="D34" s="146"/>
-      <c r="E34" s="146"/>
-      <c r="F34" s="146"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D35" s="229" t="s">
-        <v>1165</v>
-      </c>
-      <c r="E35" s="147" t="s">
-        <v>1166</v>
-      </c>
-      <c r="F35" s="229" t="s">
-        <v>1170</v>
-      </c>
-      <c r="G35" s="148" t="s">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C36" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D36" s="230" t="s">
-        <v>1168</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F36" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G36" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D37" s="232" t="str">
-        <f>D36</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F37" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D38" s="232" t="str">
-        <f t="shared" ref="D38:D41" si="0">D37</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F38" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G38" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C39" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D39" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F39" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G39" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D40" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F40" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G40" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D41" s="233" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E41" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F41" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C42" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D42" s="230" t="s">
-        <v>1174</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F42" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G42" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C43" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D43" s="232" t="str">
-        <f>D42</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F43" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G43" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C44" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D44" s="232" t="str">
-        <f t="shared" ref="D44:D47" si="1">D43</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F44" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G44" s="1">
-        <v>1.1399999999999999</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C45" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D45" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F45" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C46" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D46" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F46" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G46" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C47" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D47" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E47" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F47" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.0900000000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C48" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D48" s="230" t="s">
-        <v>1175</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F48" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G48" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C49" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D49" s="232" t="str">
-        <f>D48</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F49" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G49" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C50" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D50" s="232" t="str">
-        <f t="shared" ref="D50:D53" si="2">D49</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F50" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G50" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C51" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D51" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F51" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G51" s="1">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C52" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D52" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F52" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G52" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C53" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D53" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E53" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F53" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C54" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D54" s="230" t="s">
-        <v>1176</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F54" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G54" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C55" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D55" s="232" t="str">
-        <f>D54</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F55" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G55" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D56" s="232" t="str">
-        <f t="shared" ref="D56:D59" si="3">D55</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F56" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G56" s="1">
-        <v>1.08</v>
-      </c>
-    </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D57" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F57" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G57" s="1">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F58" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G58" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E59" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F59" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C60" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D60" s="230" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F60" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G60" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C61" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D61" s="232" t="str">
-        <f>D60</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F61" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G61" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C62" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D62" s="232" t="str">
-        <f t="shared" ref="D62:D65" si="4">D61</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F62" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G62" s="1">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C63" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D63" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F63" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G63" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C64" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D64" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F64" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C65" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D65" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E65" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F65" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G65" s="22">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F66" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G66" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated files: Enums — FID moved into -1001, LoadModelAdjustments — on load, ACCharge == 3 force-resets to "Not Verified" with a warning
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD20EB5B-36E2-4931-A02B-2BDAC4C4D805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD008B7-8B5C-4AAD-A923-959771D95CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1620" yWindow="1275" windowWidth="16575" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="1005" windowWidth="22125" windowHeight="13800" tabRatio="750" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7972" uniqueCount="1179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7862" uniqueCount="1163">
   <si>
     <t>;</t>
   </si>
@@ -3745,54 +3745,6 @@
   </si>
   <si>
     <t>09/15/25 - SAC - toggled off SysAvail for '22 VCHP Compliance Option system (gh dev #458)</t>
-  </si>
-  <si>
-    <t>NRMF 2025 ACM Table 47: HPWH System MMV (master mixing valve) Correction Factor</t>
-  </si>
-  <si>
-    <t>TABLE  T24MFDHW_CHPWH_MMVCorrectionFactor</t>
-  </si>
-  <si>
-    <t>SystemDescrip</t>
-  </si>
-  <si>
-    <t>OutletReturnDT</t>
-  </si>
-  <si>
-    <t>&lt;7</t>
-  </si>
-  <si>
-    <t>MPassInteg</t>
-  </si>
-  <si>
-    <t>Digital</t>
-  </si>
-  <si>
-    <t>MMVType</t>
-  </si>
-  <si>
-    <t>Mechanical</t>
-  </si>
-  <si>
-    <t>CorrectFactor</t>
-  </si>
-  <si>
-    <t>&gt;=7</t>
-  </si>
-  <si>
-    <t>SPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>MPassPrim-PrimTank</t>
-  </si>
-  <si>
-    <t>SPassPrim-SResist</t>
-  </si>
-  <si>
-    <t>SPassPrim-Parallel</t>
-  </si>
-  <si>
-    <t>08/01/26 - SAC - added T24MFDHW_CHPWH_MMVCorrectionFactor table (dev #942)</t>
   </si>
 </sst>
 </file>
@@ -4476,7 +4428,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="234">
+  <cellXfs count="229">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4998,21 +4950,6 @@
     <xf numFmtId="0" fontId="11" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75191,14 +75128,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="4" max="4" width="20.85546875" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
-    <col min="6" max="6" width="13.85546875" customWidth="1"/>
-    <col min="7" max="7" width="14.42578125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -75241,9 +75172,6 @@
       </c>
       <c r="B5" t="s">
         <v>3</v>
-      </c>
-      <c r="D5" t="s">
-        <v>1178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75514,602 +75442,6 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B34" s="145" t="s">
-        <v>1164</v>
-      </c>
-      <c r="C34" s="145"/>
-      <c r="D34" s="146"/>
-      <c r="E34" s="146"/>
-      <c r="F34" s="146"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="147" t="s">
-        <v>433</v>
-      </c>
-      <c r="D35" s="229" t="s">
-        <v>1165</v>
-      </c>
-      <c r="E35" s="147" t="s">
-        <v>1166</v>
-      </c>
-      <c r="F35" s="229" t="s">
-        <v>1170</v>
-      </c>
-      <c r="G35" s="148" t="s">
-        <v>1172</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C36" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D36" s="230" t="s">
-        <v>1168</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F36" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G36" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C37" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D37" s="232" t="str">
-        <f>D36</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F37" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G37" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C38" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D38" s="232" t="str">
-        <f t="shared" ref="D38:D41" si="0">D37</f>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F38" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G38" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C39" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D39" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F39" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G39" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C40" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D40" s="232" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F40" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G40" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C41" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D41" s="233" t="str">
-        <f t="shared" si="0"/>
-        <v>MPassInteg</v>
-      </c>
-      <c r="E41" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F41" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G41" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C42" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D42" s="230" t="s">
-        <v>1174</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F42" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G42" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C43" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D43" s="232" t="str">
-        <f>D42</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F43" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G43" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C44" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D44" s="232" t="str">
-        <f t="shared" ref="D44:D47" si="1">D43</f>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F44" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G44" s="1">
-        <v>1.1399999999999999</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C45" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D45" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F45" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C46" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D46" s="232" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F46" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G46" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C47" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D47" s="233" t="str">
-        <f t="shared" si="1"/>
-        <v>SPassPrim-PrimTank</v>
-      </c>
-      <c r="E47" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F47" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G47" s="22">
-        <v>1.0900000000000001</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C48" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D48" s="230" t="s">
-        <v>1175</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F48" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G48" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C49" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D49" s="232" t="str">
-        <f>D48</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F49" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G49" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C50" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D50" s="232" t="str">
-        <f t="shared" ref="D50:D53" si="2">D49</f>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F50" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G50" s="1">
-        <v>1.1499999999999999</v>
-      </c>
-    </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C51" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D51" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F51" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G51" s="1">
-        <v>0.98</v>
-      </c>
-    </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C52" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D52" s="232" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F52" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G52" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C53" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D53" s="233" t="str">
-        <f t="shared" si="2"/>
-        <v>MPassPrim-PrimTank</v>
-      </c>
-      <c r="E53" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F53" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G53" s="22">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C54" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D54" s="230" t="s">
-        <v>1176</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F54" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G54" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C55" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D55" s="232" t="str">
-        <f>D54</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F55" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G55" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C56" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D56" s="232" t="str">
-        <f t="shared" ref="D56:D59" si="3">D55</f>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F56" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G56" s="1">
-        <v>1.08</v>
-      </c>
-    </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C57" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D57" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F57" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G57" s="1">
-        <v>0.99</v>
-      </c>
-    </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C58" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D58" s="232" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F58" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G58" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C59" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D59" s="233" t="str">
-        <f t="shared" si="3"/>
-        <v>SPassPrim-SResist</v>
-      </c>
-      <c r="E59" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F59" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G59" s="22">
-        <v>1.05</v>
-      </c>
-    </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C60" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D60" s="230" t="s">
-        <v>1177</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F60" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G60" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C61" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D61" s="232" t="str">
-        <f>D60</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F61" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G61" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C62" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D62" s="232" t="str">
-        <f t="shared" ref="D62:D65" si="4">D61</f>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>1167</v>
-      </c>
-      <c r="F62" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G62" s="1">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C63" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D63" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F63" s="230" t="s">
-        <v>1169</v>
-      </c>
-      <c r="G63" s="1">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C64" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D64" s="232" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E64" s="6" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F64" s="230" t="s">
-        <v>1171</v>
-      </c>
-      <c r="G64" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C65" s="22" t="s">
-        <v>353</v>
-      </c>
-      <c r="D65" s="233" t="str">
-        <f t="shared" si="4"/>
-        <v>SPassPrim-Parallel</v>
-      </c>
-      <c r="E65" s="113" t="s">
-        <v>1173</v>
-      </c>
-      <c r="F65" s="231" t="s">
-        <v>353</v>
-      </c>
-      <c r="G65" s="22">
-        <v>1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>353</v>
-      </c>
-      <c r="F66" s="230" t="s">
-        <v>353</v>
-      </c>
-      <c r="G66" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
64-bit CSE, MF central DHW MMV and new NEEA & Central HPWH types (#1019)
* 64-bit CSE, MF central DHW MMV and new NEEA & Central HPWH types

* CSE rule mods setting ucFileName to Yes to cause CSE output to be written to All Caps filenames (as before)

* Add AnalysisResults.xml watcher to trim SF/MF UI batch storage

Parse EU-Total/EU-Compliance (SF) and TOTAL/Efficiency Compliance (MF)
metrics from AnalysisResults.xml, append to CSV, and optionally delete
Comp25/run folders and hourly sidecars while keeping XML + input models.

Co-authored-by: Demian VonderKuhlen <demian.vonderkuhlen@noresco.com>

* Revert "Add AnalysisResults.xml watcher to trim SF/MF UI batch storage"

This reverts commit f27ac5b01da52bcf934d6221cc7d661251ade6fe.

---------

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Demian VonderKuhlen <demian.vonderkuhlen@noresco.com>
</commit_message>
<xml_diff>
--- a/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
+++ b/RulesetSrc/T24SFam/To-Docu/T24R Tables.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CBECC\git-vscode\CBECC-Dev\RulesetSrc\T24SFam\To-Docu\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CD008B7-8B5C-4AAD-A923-959771D95CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD20EB5B-36E2-4931-A02B-2BDAC4C4D805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2355" yWindow="1005" windowWidth="22125" windowHeight="13800" tabRatio="750" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1620" yWindow="1275" windowWidth="16575" windowHeight="15570" tabRatio="750" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T24RClimateZoneDesignDay" sheetId="9" r:id="rId1"/>
@@ -233,7 +233,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7862" uniqueCount="1163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7972" uniqueCount="1179">
   <si>
     <t>;</t>
   </si>
@@ -3745,6 +3745,54 @@
   </si>
   <si>
     <t>09/15/25 - SAC - toggled off SysAvail for '22 VCHP Compliance Option system (gh dev #458)</t>
+  </si>
+  <si>
+    <t>NRMF 2025 ACM Table 47: HPWH System MMV (master mixing valve) Correction Factor</t>
+  </si>
+  <si>
+    <t>TABLE  T24MFDHW_CHPWH_MMVCorrectionFactor</t>
+  </si>
+  <si>
+    <t>SystemDescrip</t>
+  </si>
+  <si>
+    <t>OutletReturnDT</t>
+  </si>
+  <si>
+    <t>&lt;7</t>
+  </si>
+  <si>
+    <t>MPassInteg</t>
+  </si>
+  <si>
+    <t>Digital</t>
+  </si>
+  <si>
+    <t>MMVType</t>
+  </si>
+  <si>
+    <t>Mechanical</t>
+  </si>
+  <si>
+    <t>CorrectFactor</t>
+  </si>
+  <si>
+    <t>&gt;=7</t>
+  </si>
+  <si>
+    <t>SPassPrim-PrimTank</t>
+  </si>
+  <si>
+    <t>MPassPrim-PrimTank</t>
+  </si>
+  <si>
+    <t>SPassPrim-SResist</t>
+  </si>
+  <si>
+    <t>SPassPrim-Parallel</t>
+  </si>
+  <si>
+    <t>08/01/26 - SAC - added T24MFDHW_CHPWH_MMVCorrectionFactor table (dev #942)</t>
   </si>
 </sst>
 </file>
@@ -4428,7 +4476,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="229">
+  <cellXfs count="234">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4950,6 +4998,21 @@
     <xf numFmtId="0" fontId="11" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
@@ -75128,8 +75191,14 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:G68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="20.85546875" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="14.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -75172,6 +75241,9 @@
       </c>
       <c r="B5" t="s">
         <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1178</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -75442,6 +75514,602 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B34" s="145" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C34" s="145"/>
+      <c r="D34" s="146"/>
+      <c r="E34" s="146"/>
+      <c r="F34" s="146"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C35" s="147" t="s">
+        <v>433</v>
+      </c>
+      <c r="D35" s="229" t="s">
+        <v>1165</v>
+      </c>
+      <c r="E35" s="147" t="s">
+        <v>1166</v>
+      </c>
+      <c r="F35" s="229" t="s">
+        <v>1170</v>
+      </c>
+      <c r="G35" s="148" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C36" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D36" s="230" t="s">
+        <v>1168</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F36" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G36" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C37" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D37" s="232" t="str">
+        <f>D36</f>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F37" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G37" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C38" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D38" s="232" t="str">
+        <f t="shared" ref="D38:D41" si="0">D37</f>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F38" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G38" s="1">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C39" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D39" s="232" t="str">
+        <f t="shared" si="0"/>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F39" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G39" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C40" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D40" s="232" t="str">
+        <f t="shared" si="0"/>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F40" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G40" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C41" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="D41" s="233" t="str">
+        <f t="shared" si="0"/>
+        <v>MPassInteg</v>
+      </c>
+      <c r="E41" s="113" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F41" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G41" s="22">
+        <v>1.1200000000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C42" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D42" s="230" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F42" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G42" s="1">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C43" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D43" s="232" t="str">
+        <f>D42</f>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F43" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G43" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C44" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D44" s="232" t="str">
+        <f t="shared" ref="D44:D47" si="1">D43</f>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F44" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G44" s="1">
+        <v>1.1399999999999999</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C45" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D45" s="232" t="str">
+        <f t="shared" si="1"/>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F45" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G45" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C46" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D46" s="232" t="str">
+        <f t="shared" si="1"/>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F46" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G46" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C47" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="D47" s="233" t="str">
+        <f t="shared" si="1"/>
+        <v>SPassPrim-PrimTank</v>
+      </c>
+      <c r="E47" s="113" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F47" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G47" s="22">
+        <v>1.0900000000000001</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C48" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D48" s="230" t="s">
+        <v>1175</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F48" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G48" s="1">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C49" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D49" s="232" t="str">
+        <f>D48</f>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F49" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G49" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C50" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D50" s="232" t="str">
+        <f t="shared" ref="D50:D53" si="2">D49</f>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F50" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G50" s="1">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C51" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D51" s="232" t="str">
+        <f t="shared" si="2"/>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F51" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G51" s="1">
+        <v>0.98</v>
+      </c>
+    </row>
+    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C52" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D52" s="232" t="str">
+        <f t="shared" si="2"/>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F52" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G52" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C53" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="D53" s="233" t="str">
+        <f t="shared" si="2"/>
+        <v>MPassPrim-PrimTank</v>
+      </c>
+      <c r="E53" s="113" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F53" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G53" s="22">
+        <v>1.1200000000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C54" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D54" s="230" t="s">
+        <v>1176</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F54" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G54" s="1">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C55" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D55" s="232" t="str">
+        <f>D54</f>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F55" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G55" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C56" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D56" s="232" t="str">
+        <f t="shared" ref="D56:D59" si="3">D55</f>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F56" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G56" s="1">
+        <v>1.08</v>
+      </c>
+    </row>
+    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C57" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D57" s="232" t="str">
+        <f t="shared" si="3"/>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F57" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G57" s="1">
+        <v>0.99</v>
+      </c>
+    </row>
+    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C58" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D58" s="232" t="str">
+        <f t="shared" si="3"/>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F58" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G58" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C59" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="D59" s="233" t="str">
+        <f t="shared" si="3"/>
+        <v>SPassPrim-SResist</v>
+      </c>
+      <c r="E59" s="113" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F59" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G59" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C60" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D60" s="230" t="s">
+        <v>1177</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F60" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G60" s="1">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C61" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D61" s="232" t="str">
+        <f>D60</f>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F61" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G61" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C62" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D62" s="232" t="str">
+        <f t="shared" ref="D62:D65" si="4">D61</f>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>1167</v>
+      </c>
+      <c r="F62" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G62" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C63" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D63" s="232" t="str">
+        <f t="shared" si="4"/>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F63" s="230" t="s">
+        <v>1169</v>
+      </c>
+      <c r="G63" s="1">
+        <v>0.96</v>
+      </c>
+    </row>
+    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="C64" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D64" s="232" t="str">
+        <f t="shared" si="4"/>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F64" s="230" t="s">
+        <v>1171</v>
+      </c>
+      <c r="G64" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C65" s="22" t="s">
+        <v>353</v>
+      </c>
+      <c r="D65" s="233" t="str">
+        <f t="shared" si="4"/>
+        <v>SPassPrim-Parallel</v>
+      </c>
+      <c r="E65" s="113" t="s">
+        <v>1173</v>
+      </c>
+      <c r="F65" s="231" t="s">
+        <v>353</v>
+      </c>
+      <c r="G65" s="22">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C66" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F66" s="230" t="s">
+        <v>353</v>
+      </c>
+      <c r="G66" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>